<commit_message>
Update Kappa method using desc corpus
</commit_message>
<xml_diff>
--- a/data/Anotasi Skill - Gopal.xlsx
+++ b/data/Anotasi Skill - Gopal.xlsx
@@ -2,33 +2,29 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Posting" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SFIA" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Evaluasi" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -42,27 +38,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -75,22 +56,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -163,20 +138,20 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Sheets">
+    <a:clrScheme name="Office">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="000000"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="4F81BD"/>
@@ -200,19 +175,77 @@
         <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Sheets">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -224,131 +257,160 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -364,58 +426,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Nama Pekerjaan</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Deskripsi Pekerjaan</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Hasil Ekstraksi Sistem</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Hasil Anotasi Pakar</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>TP</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>FP</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>FN</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Precision</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>F1-Score</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Korpus</t>
         </is>
       </c>
     </row>
@@ -504,6 +571,11 @@
       </c>
       <c r="J2" t="n">
         <v>0.6829</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>minimum education graduates prioritized department information engineering information systems related fields mastering c # programming language java php understand experience developing erp enterprise resource planning system experience involved projects related erp mastering sql database example mysql sql server postgresql able write queries manage databases work experience project relevant development erp based applications understand concept oop object oriented programming familiar development tools git visual studio related ideas able work team good communication</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -617,6 +689,11 @@
       <c r="J3" t="n">
         <v>0.6071</v>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>design develop implement comprehensive test scenarios scripts ensure overall product quality execute manual automated testing identify bugs system defects inconsistencies analyze test outcomes compile detailed bug reports actionable recommendations improvements perform thorough regression testing following system fixes updates ensure functionality stability collaborate closely development teams understand technical specifications business requirements contribute design aesthetically pleasing responsive user friendly user interfaces ui conduct usability testing refine designs based test results user feedback candidates must hold minimum diploma bachelor degree computer science information technology related field previous experience quality assurance software/application testing highly preferred strong understanding manual automated testing methodologies advantageous experience qa tools selenium appium postman plus demonstrates strong critical thinking analytical problem solving abilities familiarity ui/ux design principles usability testing plus fluency indonesian english required proactive responsible individual strong sense ownership must possess personal vehicle valid driver license applicants older years age</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -716,6 +793,11 @@
       <c r="J4" t="n">
         <v>0.5659999999999999</v>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>minimum information technology engineering computer science/related proficient object oriented programming asp net sql knowledge development using c # asp net mvc razor html knowledge web services wcf rest soap etc web api sql able develop using application lifecycle management tools vsts/git knowledge javascript jquery css angularjs telerik plus self motivated takes accountability ownership work minimum supervision fresh graduates want unleash potential net developer welcome apply mcsd web application certification advantage</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -791,6 +873,11 @@
       </c>
       <c r="J5" t="n">
         <v>0.7333</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>develop quality software web applications analyze maintain existing software applications design highly scalable testable code discover fix programming bugs bachelor degree equivalent experience computer science related field development experience programming languages sql database relational database skills curiosity ability quickly adapt emerging ai technologies familiar ai libraries frameworks</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -881,6 +968,11 @@
       <c r="J6" t="n">
         <v>0.6667</v>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>process analyze data deliver accurate timely routine ad hoc reports enhance data processing analysis workflow based best practices actively support execute various initiatives meet business management needs facilitate user requests reporting analytical enhancements bachelor degree management business accounting information systems industrial engineering relevant fields fresh graduate year experience data analysis background excellent microsoft excel experience excel macros/vba strong value added proficient communication skills english written verbal demonstrated ability manage multiple tasks prioritize effectively work collaboratively cross functional teams willing placed jakarta/cibitung</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -957,6 +1049,11 @@
       </c>
       <c r="J7" t="n">
         <v>0.7272999999999999</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>bachelor degree majoring informatic engineering / computer science / information system / major related minimum years working experience web app / mobile app development / backend developer would advantage ; fresh graduates welcome apply able work independently team &amp; familiar dealing collaborating departments / cross functional teams excellent analytical &amp; time management skills willing placed kitic cikarang design builds maintain scalable secure high performance server side applications apis databases deliver digital seamless digital experiences adhering best practices coding security system architecture</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -1040,6 +1137,11 @@
       </c>
       <c r="J8" t="n">
         <v>0.7895</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>building robust large scale social media crawler various social media platforms maintain day day operation said crawlers alongside data quality team make sure completeness timeliness incoming data work team along several stakeholders better understand communicate data requirements issues intermediate advanced understanding sql proficiency several programming languages mainly javascript node python good experience using scala production related spark big plus intermediate advanced understanding several data related technologies mariadb postgres redis kafka elasticsearch ample experience using linux based system understanding several data acquisition techniques webscraping api based data consumption</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -1137,6 +1239,11 @@
       </c>
       <c r="J9" t="n">
         <v>0.8260999999999999</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>fresh graduate maximum years experience auditing governance risk management compliance network security minimum bachelor ’ degree information technology computer science information systems cybersecurity information security minimum gpa strong knowledge systems software programming system control familiarity penetration testing methodologies tools excellent communication interpersonal skills high analytical skills proactive approach problem solving understanding auditing principles practice highly preferred conduct audits systems processes ensure compliance internal policies external regulations evaluate effectiveness controls identify areas improvement collaborate teams understand software programming system control mechanisms prepare detailed audit reports clearly communicate findings recommendations management conduct risk assessment analyze system vulnerabilities stay updated industry trends best practices emerging technologies related auditing</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1241,6 +1348,11 @@
       <c r="J10" t="n">
         <v>0.6038</v>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>design develop deploy machine learning models pipelines various business use cases preprocess clean validate large datasets use training inference conduct research stay updated latest ai/ml trends frameworks best practices optimize models performance scalability efficiency collaborate data engineers software developers integrate ml models production systems monitor model performance retrain models needed document work write clean maintainable code follow best practices software development mlops proficient python ml frameworks e g tensorflow pytorch scikit learn solid understanding machine learning deep learning concepts experience data preprocessing model deployment familiar git ; docker mlops tools plus strong problem solving teamwork skills bachelor ’ computer science related field</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1319,6 +1431,11 @@
       </c>
       <c r="J11" t="n">
         <v>0.8235</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>least year experience developer fresh graduates final year students invited apply experiences rdbms postgresql ms sql server mysql good understanding git version control system familiar agile/scrum methodology supporting tools experience message brokers rabbitmq kafka added value analytical abilities problem solving strong troubleshooting good communication skills effective collaboration team minimum diploma bachelor education fields computer science engineering related fields take precedence</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1434,6 +1551,11 @@
       <c r="J12" t="n">
         <v>0.6</v>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>design develop web backend services using django framework python write high quality clean maintainable code using engineering best practices unit testing source control git continuous integration automation design patterns etc analyze requirements design develop features understand product continuously optimize address issues enhance stability user experience optimize applications achieve maximum performance scalability create reusable code libraries future use collaborate fellow developers product managers build products web technologies minimum bachelor degree computer science related fields years working experience fresh graduates relevant internship experiences welcome apply passionate coding programming innovation solving challenging problems hands experiences web service frameworks technologies django &amp; python sql nosql familiar http protocol skilled handling cache &amp; database logic understanding data structures computer science fundamentals familiar linux development environments experience key value databases like redis memcached plus knowledge fastapi added advantage willing work months fixed term employment office south jakarta</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1531,6 +1653,11 @@
       </c>
       <c r="J13" t="n">
         <v>0.5652</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>fresh graduate maximum years experience sysadmin / operations / infrastructure fields work minimum bachelor ’ degree information technology software engineering informatics engineering minimum gpa understanding systems processes strong technical knowledge network server operating system good knowledge scripting cli sql programming basic knowledge data security cyber security basics vast experience mikrotik switches vm ha enterprise backup solution oversees maintains aspects company infrastructure including performances health automate backup operational levels responsible ensuring smooth operations systems including networks firewalls ip segments etc hardwares development networking security devices servers vps baremetal offshore backups services may include third party software and/or developed contributing development department policies scalability coordinate internal department services provided company act l support make smooth transition l services operated company providing guide documented troubleshoot procedure contribute related project liaise vendors coordinate superior perform duties assigned supervisor support infrastructure efficiency development</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -1648,6 +1775,11 @@
       <c r="J14" t="n">
         <v>0.6102</v>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>bachelor ’ degree computer science statistics information systems related field proven experience data analyst bi engineer similar role strong proficiency sql experience relational databases experience bi tools power bi tableau looker similar platforms familiarity data warehousing concepts etl processes solid understanding data modeling data architecture data governance excellent problem solving skills attention detail strong communication skills capable explaining complex data insights non technical stakeholders willing placed ho balikpapan representative office jakarta collect process analyze large datasets multiple sources identify trends patterns opportunities design develop maintain dashboards reports visualizations using bi tools e g superset power bi tableau looker collaborate stakeholders understand business requirements translate technical specifications develop optimize sql queries data pipelines extract transform data efficiently ensure data accuracy integrity consistency across reporting platforms perform root cause analysis data discrepancies troubleshoot data related issues automate repetitive reporting tasks optimize existing workflows provide actionable insights recommendations based data analysis support business decisions stay updated latest bi trends tools best practices ability work agile development environment strong business acumen ability align bi solutions organizational goals</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1744,6 +1876,11 @@
       <c r="J15" t="n">
         <v>0.7727000000000001</v>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>analyse design develop apps based customer business bank operational needs perform system testing unit tests system integration tests ensure application used connected required systems monitor maintain apps performance enhancement suit needs customers business bank operations develop manage documentation related apps development experience handling core loan prioritized familiar java years experience core banking preferable good understanding microservice api familiar agile scrum framework familiar postgresql mysql database good communication collaboration skill good understanding software security able code testing bug troubleshooting provide application support updated technological developments fresh graduate welcome apply</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1809,6 +1946,11 @@
       </c>
       <c r="J16" t="n">
         <v>0.8</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>software testing qa testing bug tracking skills experience test case creation knowledge software development lifecycle testing methodologies experience test automation tools analytical problem solving skills excellent attention detail organizational skills ability work independently remotely pursuing degree computer science information technology related field previous internship experience software testing plus</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1881,6 +2023,11 @@
       </c>
       <c r="J17" t="n">
         <v>0.4762</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>fluent spoken written english good understanding basic technical terms experience desktop support online &amp; offline knowledge cloud technology security plus willing support various functions projects must available join immediately hardware support : inventory installation upgrades troubleshooting software support : installation testing issue resolution network support : inventory vendor coordination troubleshooting business support : user support sla tracking ticket handling project support : assist related project execution competitive salary + overtime pay hands involvement various projects exposure latest technologies tools</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1978,6 +2125,11 @@
       <c r="J18" t="n">
         <v>0.6842</v>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>conduct user research understand needs problems user behavior collect analyze user data interviews surveys ux test results creating clear functional low fidelity high fidelity wireframes using figma develop interactive prototype initial testing concept presentation designing interface responsive aesthetic accordance company brand identity using modern design principles visual hierarchy consistency good typography collaborated closely development team ensure implementation design runs according plan provide design specifications style guidelines technical team usability testing identify repair area implement feedback users teams perfect design creating maintaining design system including reusable component figure documenting design decisions workflows team references figma main adobe illustrator optional canva optional make design good ui/ux oriented detail quality high responsibility &amp; consistency ability work together teams fast adapting &amp; learning new things</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2045,6 +2197,11 @@
       </c>
       <c r="J19" t="n">
         <v>0.5</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>concept create professional web design engag meet company brand continuously improve optimize user experience exploring company website collaborated developing concepts design ideas divisions marketing customer relationship management smk/d/d/s field information engineering communication information technology mandatory familiar html css javascript mandatory familiar wordpress able use graphic design tools</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -2131,6 +2288,11 @@
       <c r="J20" t="n">
         <v>0.4</v>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>working alongside tech &amp; product team develop engaging &amp; responsive user interfaces html css modern javascript frameworks experience angular frontend flutter mobile java spring boot framework backend develop performance oriented front end &amp; back end binding work back end developers design interface rest apis perform code reviews basic troubleshooting build reusable code libraries future use minimum years experience experience full stack development whether house agency freelancer bachelor degree computer science information technology equivalent managing multiple tasks timelines fast paced environment experience team leader plus humility excellent collaborative spirit learn grow together team fresh graduates prior intern/project experience angular flutter java spring boot welcome apply thr / bpjs ketenagakerjaan / bpjs kesehatan / private insurance / glasses allowance</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2198,6 +2360,11 @@
       <c r="J21" t="n">
         <v>0.4545</v>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>conduct operation monitoring within customer provide st level support external customer perform network troubleshooting customer conduct operation &amp; security monitoring within customer bachelor degree computer engineering electrical engineering computer science/information technology equivalent experience technical support engineer similar role skill network routing switching cisco product switch meraki placement south jakarta</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2210,58 +2377,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Skill - Level</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Deskripsi Level</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Hasil Ekstraksi Sistem</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Hasil Anotasi Pakar</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>TP</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>FP</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>FN</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Precision</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Recall</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>F1-Score</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Korpus</t>
         </is>
       </c>
     </row>
@@ -2317,6 +2489,11 @@
       <c r="J2" t="n">
         <v>0.6667</v>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>designs codes verifies tests documents amends refactors complex programs/scripts integration software services contributes selection software development methods tools techniques security practices applies agreed standards tools security measures achieve well engineered outcomes participates reviews work leads reviews colleagues work</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2371,6 +2548,11 @@
       </c>
       <c r="J3" t="n">
         <v>0.8571</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>champions leads introduction use data science drive innovation business value develops drives adoption adherence organisational policies standards guidelines methods data science sets direction leads introduction use data science techniques methodologies tools leads development organisational capabilities data science plans leads strategic large complex data science initiatives generate insights create value drive decision making</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -2434,6 +2616,11 @@
       <c r="J4" t="n">
         <v>0.6667</v>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>assesses suitability machine learning designs develops solutions range business problems selects applies appropriate techniques algorithms based data characteristics business requirements provides guidance others engineers features optimises model performance implements algorithms contributes development evaluation monitoring deployment applies industry specific rules guidelines anticipating risks implications collaborates cross functional teams integrate machine learning models production systems conducts depth performance analysis troubleshoots issues</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2493,6 +2680,11 @@
       </c>
       <c r="J5" t="n">
         <v>0.8421</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>directs creation review cross functional enterprise wide approach culture generating value data analytics data science drives identification evaluation adoption data analytics data science capabilities transform organisational performance leads provision organisation ’ data analytics data science capabilities ensures strategic application data analytics data science embedded governance leadership organisation aligns business strategies enterprise transformation data analytics data science strategies</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -2556,6 +2748,11 @@
       <c r="J6" t="n">
         <v>0.8571</v>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>designs implements maintains complex data engineering solutions acquire prepare data creates maintains data pipelines connect data across data stores applications organisations builds compliance data governance security standards supports development continuous integration deployment practices monitors optimises pipeline performance scalability conducts complex data quality checking remediation leads data migration data conversion activities</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2615,6 +2812,11 @@
       </c>
       <c r="J7" t="n">
         <v>0.6316000000000001</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>leads exploration new approaches data visualisation establishes purpose parameters data visualisation oversees use data visualisation tools techniques communicates results using appropriate methods target audience advises use data visualisation approaches different purposes contexts satisfy requirements develops plans meet user needs collaborates stakeholders identify key insights create compelling narratives effectively communicate story behind data drive decision making processes</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -2681,6 +2883,11 @@
       <c r="J8" t="n">
         <v>0.75</v>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>designs visual concepts comprehensive designs complex assignments engages clients stakeholders elicit document design requirements goals manages design assignments concept final delivery creates detailed design mock ups interactive prototypes reviews approves design work ensuring alignment brand standards evidence based practices develops implements design processes guidelines recognised good practices enhance design quality effectiveness</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2736,6 +2943,11 @@
       <c r="J9" t="n">
         <v>0.7143</v>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>responsible operation incident management process manages incident communications ensuring al parties aware incidents role process leads review major incidents informs service owners outcomes ensures incident resolution within service targets analyses metrics reports performance incident management process develops maintains tests incident management policy procedures ensures compliance regulatory requirements</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2787,6 +2999,11 @@
       </c>
       <c r="J10" t="n">
         <v>0.7272999999999999</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>plans drives penetration testing within defined area business activity delivers objective insights existence vulnerabilities effectiveness defences mitigating controls takes responsibility integrity testing activities coordinates execution activities provides authoritative advice guidance aspects penetration testing identifies needs implements new approaches penetration testing contributes security testing standards</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -2854,6 +3071,11 @@
       <c r="J11" t="n">
         <v>0.5833</v>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>takes full responsibility definition approach facilitation satisfactory completion medium scale projects provides effective leadership project team adopting suitable project management methods tools manages change control processes assesses risks ensuring projects align governance frameworks business priorities communicates regularly stakeholders ensuring project deliverables meet agreed standards budgets timelines ensures project product quality reviews occur schedule according procedure proactively monitors performance metrics implementing preventive corrective actions needed</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2906,6 +3128,11 @@
       </c>
       <c r="J12" t="n">
         <v>0.3333</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>plans organises conducts formal reviews assessments complex domains areas cross functional areas across supply chain evaluates appraises identifies non compliances organisational standards determines underlying reasons non compliance prepares reports assessment findings associated risks ensures appropriate owners corrective actions identified identifies opportunities improve organisational control mechanisms oversees assurance activities others providing advice expertise support assurance activity</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -2969,6 +3196,11 @@
       <c r="J13" t="n">
         <v>0.8182</v>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>plans manages implementation organisation wide risk management processes integrating tools techniques aligned governance frameworks considers organisation wide risk mitigation activities within context business risk whole organisation ’ appetite risk provides leadership risk management ensuring practices support strategic decision making compliance organisational policies</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3032,6 +3264,11 @@
       <c r="J14" t="n">
         <v>0.7619</v>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>designs system components using appropriate modelling techniques following agreed architectures design standards patterns methodology identifies evaluates alternative design options trade offs creates multiple design views address concerns different stakeholders handle functional non functional requirements models simulates prototypes behaviour proposed system components enable approval stakeholders produces detailed design specifications form basis construction systems reviews verifies improves designs specifications</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3092,6 +3329,11 @@
       </c>
       <c r="J15" t="n">
         <v>0.6</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>specifies designs architects large complex software applications components modules adopts adapts software design methods tools techniques undertakes impact analysis major design options makes recommendations assesses manages associated risks specifies prototypes/simulations enable informed decision making evaluates software designs ensure adherence standards identifies corrective action ensures software design balances functional quality security systems management requirements contributes development organisational software design architecture policies standards</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -3156,6 +3398,11 @@
       <c r="J16" t="n">
         <v>0.7272999999999999</v>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>designs specific network components using agreed architectures design standards patterns methodology translates logical designs physical designs meet specified operational parameters capacity performance reviews verifies network designs non functional requirements including validation error correction procedures access security audit controls contributes development recovery routines contingency procedures contributes alternative network architectures networking topologies design options</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3219,6 +3466,11 @@
       <c r="J17" t="n">
         <v>0.6364</v>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>develops communicates corporate information security policy standards guidelines ensures architectural principles applied design reduce risk drives adoption adherence policy standards guidelines contributes development organisational strategies address information control requirements identifies monitors environmental market trends proactively assesses impact business strategies benefits risks leads provision authoritative advice guidance requirements security controls collaboration subject matter experts</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3273,6 +3525,11 @@
       </c>
       <c r="J18" t="n">
         <v>0.5714</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>engages stakeholders communicate ethical considerations influence design decisions conducts detailed impact assessments makes recommendations manages ethical reviews ensure compliance standards evaluates risks proposes measures address ethical concerns leads discussions stakeholders ethical issues designs executes ethical impact assessments prepares reports based audit findings</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -3336,6 +3593,11 @@
       <c r="J19" t="n">
         <v>0.8571</v>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>plans organises conducts audits complex domains areas cross functional areas across supply chain confirms scope objectives specific audit activities management aligns scope audit programme organisational policies determines appropriate methods investigation achieve audit objectives presents audit findings management describing effectiveness efficiency control mechanisms provides general specific audit advice collaborates professionals related specialisms develop integrate findings</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3388,6 +3650,11 @@
       </c>
       <c r="J20" t="n">
         <v>0.7692</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>develops organisational policies standards guidelines software configuration design deployment refactoring plans leads software configuration deployment activities strategic large complex deployment projects develops new methods organisational capabilities drives adoption adherence policies standards</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -3446,106 +3713,10 @@
       <c r="J21" t="n">
         <v>0.8235</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Sheet</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Total TP</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Total FP</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Total FN</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Avg Precision</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Avg Recall</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Avg F1-Score</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Job Posting</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>257</v>
-      </c>
-      <c r="C2" t="n">
-        <v>162</v>
-      </c>
-      <c r="D2" t="n">
-        <v>119</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.6196</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.6843</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.6445</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>SFIA</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>130</v>
-      </c>
-      <c r="C3" t="n">
-        <v>56</v>
-      </c>
-      <c r="D3" t="n">
-        <v>47</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.7123</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.7284</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.7097</v>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>provides specialist expertise design characteristics database management systems data warehouse products/services provides expert guidance selection provision use database data warehouse architectures software facilities ensures design policies optimise transactional data systems performance availability meeting needs business intelligence analytics platforms</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>